<commit_message>
Prepare saints seed for production review
</commit_message>
<xml_diff>
--- a/supabase-connect-main/supabase/seed/saints/published/Doctors-Pack-01.xlsx
+++ b/supabase-connect-main/supabase/seed/saints/published/Doctors-Pack-01.xlsx
@@ -523,7 +523,7 @@
         <v>Romans 13:13-14</v>
       </c>
       <c r="S2" t="str">
-        <v>doctor of the church,bishop,theologian,conversion,north africa,grace</v>
+        <v>doctor-of-the-church,bishop,theologian,conversion,north-africa,grace</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -591,7 +591,7 @@
         <v>2 Timothy 3:16-17</v>
       </c>
       <c r="S3" t="str">
-        <v>doctor of the church,priest,scripture,translator,bible,scholar,monastic</v>
+        <v>doctor-of-the-church,priest,scripture,translator,bible,scholar,monastic</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -659,7 +659,7 @@
         <v>John 10:11</v>
       </c>
       <c r="S4" t="str">
-        <v>doctor of the church,bishop,milan,preacher,orthodoxy,leadership</v>
+        <v>doctor-of-the-church,bishop,milan,preacher,orthodoxy,leadership</v>
       </c>
       <c r="T4" t="b">
         <v>1</v>
@@ -727,7 +727,7 @@
         <v>1 Peter 5:2-4</v>
       </c>
       <c r="S5" t="str">
-        <v>doctor of the church,pope,pastor,missionary,monastic,teacher</v>
+        <v>doctor-of-the-church,pope,pastor,missionary,monastic,teacher</v>
       </c>
       <c r="T5" t="b">
         <v>1</v>
@@ -795,7 +795,7 @@
         <v>Wisdom 7:7-10</v>
       </c>
       <c r="S6" t="str">
-        <v>doctor of the church,priest,dominican,theologian,philosopher,eucharist,teacher</v>
+        <v>doctor-of-the-church,priest,dominican,theologian,philosopher,eucharist,teacher</v>
       </c>
       <c r="T6" t="b">
         <v>1</v>

</xml_diff>